<commit_message>
feat: Introduce a new user and access role management module and add administrative configuration modals to the health flow interface.
</commit_message>
<xml_diff>
--- a/Price_List_Adjustments_Rules_20250921 V4.0 Scrubbed.xlsx
+++ b/Price_List_Adjustments_Rules_20250921 V4.0 Scrubbed.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9303"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11028"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adity/Documents/GitHub/health19/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81ADBF2A-7959-D546-901C-40A9BAD41136}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="20" windowWidth="16100" windowHeight="9660" activeTab="1"/>
+    <workbookView xWindow="240" yWindow="500" windowWidth="36000" windowHeight="20600" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hanoi_Adjustments_Clean" sheetId="1" r:id="rId1"/>
@@ -12,12 +18,24 @@
     <sheet name="Hanoi_Base_Clean_v3" sheetId="3" r:id="rId3"/>
     <sheet name="HCMC_Base_Clean_v3" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="145621"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2728" uniqueCount="467">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2756" uniqueCount="467">
   <si>
     <t>Region</t>
   </si>
@@ -1423,7 +1441,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1476,12 +1494,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -1498,14 +1515,17 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1543,7 +1563,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -1615,7 +1635,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1788,26 +1808,26 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:P35"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="6.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="37.26953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="53.26953125" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="53.26953125" customWidth="1"/>
-    <col min="6" max="6" width="49.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="37.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="53.33203125" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="53.33203125" customWidth="1"/>
+    <col min="6" max="6" width="49.5" bestFit="1" customWidth="1"/>
     <col min="7" max="8" width="17" customWidth="1"/>
-    <col min="9" max="10" width="24.26953125" customWidth="1"/>
-    <col min="11" max="11" width="48.1796875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.1796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="24.33203125" customWidth="1"/>
+    <col min="11" max="11" width="48.1640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.1640625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="35" customWidth="1"/>
-    <col min="14" max="14" width="24.08984375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="24.08984375" customWidth="1"/>
-    <col min="16" max="16" width="34.54296875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="24.1640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="24.1640625" customWidth="1"/>
+    <col min="16" max="16" width="34.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1857,7 +1877,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1904,7 +1924,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -1951,7 +1971,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -1998,7 +2018,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -2045,7 +2065,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -2092,7 +2112,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -2139,7 +2159,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -2189,7 +2209,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -2239,7 +2259,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>4</v>
       </c>
@@ -2289,7 +2309,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>4</v>
       </c>
@@ -2339,7 +2359,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -2389,7 +2409,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>4</v>
       </c>
@@ -2439,7 +2459,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>4</v>
       </c>
@@ -2489,7 +2509,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>4</v>
       </c>
@@ -2539,7 +2559,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>4</v>
       </c>
@@ -2589,7 +2609,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>4</v>
       </c>
@@ -2639,7 +2659,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>4</v>
       </c>
@@ -2689,7 +2709,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>4</v>
       </c>
@@ -2739,7 +2759,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>4</v>
       </c>
@@ -2789,7 +2809,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>4</v>
       </c>
@@ -2839,7 +2859,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>4</v>
       </c>
@@ -2889,7 +2909,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>4</v>
       </c>
@@ -2939,7 +2959,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>4</v>
       </c>
@@ -2989,7 +3009,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>4</v>
       </c>
@@ -3039,7 +3059,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>4</v>
       </c>
@@ -3089,7 +3109,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>4</v>
       </c>
@@ -3139,7 +3159,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>4</v>
       </c>
@@ -3189,7 +3209,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>4</v>
       </c>
@@ -3239,7 +3259,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>4</v>
       </c>
@@ -3289,7 +3309,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>4</v>
       </c>
@@ -3339,7 +3359,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>4</v>
       </c>
@@ -3389,7 +3409,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>4</v>
       </c>
@@ -3439,7 +3459,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>4</v>
       </c>
@@ -3489,7 +3509,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>4</v>
       </c>
@@ -3545,27 +3565,27 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:P124"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="6.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="26.90625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="54.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="54.36328125" customWidth="1"/>
+    <col min="1" max="1" width="6.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="54.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="54.33203125" customWidth="1"/>
     <col min="6" max="6" width="64" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.26953125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.54296875" customWidth="1"/>
-    <col min="9" max="9" width="17.90625" bestFit="1" customWidth="1"/>
-    <col min="10" max="11" width="48.1796875" customWidth="1"/>
-    <col min="12" max="12" width="8.1796875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="27.36328125" customWidth="1"/>
-    <col min="14" max="14" width="33.08984375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="33.08984375" customWidth="1"/>
-    <col min="16" max="16" width="48.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.5" customWidth="1"/>
+    <col min="9" max="9" width="17.83203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="48.1640625" customWidth="1"/>
+    <col min="12" max="12" width="8.1640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="27.33203125" customWidth="1"/>
+    <col min="14" max="14" width="33.1640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="33.1640625" customWidth="1"/>
+    <col min="16" max="16" width="48.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3615,7 +3635,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>91</v>
       </c>
@@ -3666,7 +3686,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>91</v>
       </c>
@@ -3717,7 +3737,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>91</v>
       </c>
@@ -3768,7 +3788,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>91</v>
       </c>
@@ -3819,7 +3839,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>91</v>
       </c>
@@ -3870,7 +3890,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>91</v>
       </c>
@@ -3921,7 +3941,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>91</v>
       </c>
@@ -3972,7 +3992,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>91</v>
       </c>
@@ -4023,7 +4043,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>91</v>
       </c>
@@ -4074,7 +4094,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>91</v>
       </c>
@@ -4125,7 +4145,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>91</v>
       </c>
@@ -4176,7 +4196,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>91</v>
       </c>
@@ -4227,7 +4247,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>91</v>
       </c>
@@ -4278,7 +4298,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>91</v>
       </c>
@@ -4329,7 +4349,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>91</v>
       </c>
@@ -4380,7 +4400,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>91</v>
       </c>
@@ -4431,7 +4451,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>91</v>
       </c>
@@ -4482,7 +4502,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>91</v>
       </c>
@@ -4533,7 +4553,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>91</v>
       </c>
@@ -4584,7 +4604,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>91</v>
       </c>
@@ -4635,7 +4655,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>91</v>
       </c>
@@ -4686,7 +4706,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>91</v>
       </c>
@@ -4737,7 +4757,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>91</v>
       </c>
@@ -4788,7 +4808,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>91</v>
       </c>
@@ -4839,7 +4859,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>91</v>
       </c>
@@ -4890,7 +4910,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>91</v>
       </c>
@@ -4941,7 +4961,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>91</v>
       </c>
@@ -4992,7 +5012,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>91</v>
       </c>
@@ -5043,7 +5063,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>91</v>
       </c>
@@ -5094,7 +5114,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>91</v>
       </c>
@@ -5145,7 +5165,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>91</v>
       </c>
@@ -5196,7 +5216,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>91</v>
       </c>
@@ -5247,7 +5267,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>91</v>
       </c>
@@ -5298,7 +5318,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>91</v>
       </c>
@@ -5349,7 +5369,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>91</v>
       </c>
@@ -5400,7 +5420,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>91</v>
       </c>
@@ -5451,7 +5471,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>91</v>
       </c>
@@ -5502,7 +5522,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>91</v>
       </c>
@@ -5552,7 +5572,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>91</v>
       </c>
@@ -5602,7 +5622,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>91</v>
       </c>
@@ -5652,7 +5672,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>91</v>
       </c>
@@ -5702,7 +5722,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>91</v>
       </c>
@@ -5752,7 +5772,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>91</v>
       </c>
@@ -5799,7 +5819,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>91</v>
       </c>
@@ -5846,7 +5866,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>91</v>
       </c>
@@ -5893,7 +5913,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>91</v>
       </c>
@@ -5940,7 +5960,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>91</v>
       </c>
@@ -5987,7 +6007,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="49" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>91</v>
       </c>
@@ -6037,7 +6057,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="50" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>91</v>
       </c>
@@ -6087,7 +6107,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="51" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>91</v>
       </c>
@@ -6137,7 +6157,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="52" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>91</v>
       </c>
@@ -6187,7 +6207,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="53" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>91</v>
       </c>
@@ -6237,7 +6257,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="54" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>91</v>
       </c>
@@ -6287,7 +6307,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="55" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>91</v>
       </c>
@@ -6337,7 +6357,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>91</v>
       </c>
@@ -6387,7 +6407,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="57" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>91</v>
       </c>
@@ -6437,7 +6457,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="58" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>91</v>
       </c>
@@ -6487,7 +6507,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="59" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>91</v>
       </c>
@@ -6537,7 +6557,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="60" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>91</v>
       </c>
@@ -6587,7 +6607,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="61" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>91</v>
       </c>
@@ -6637,7 +6657,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="62" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>91</v>
       </c>
@@ -6687,7 +6707,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="63" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>91</v>
       </c>
@@ -6737,7 +6757,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="64" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>91</v>
       </c>
@@ -6787,7 +6807,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="65" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>91</v>
       </c>
@@ -6837,7 +6857,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="66" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>91</v>
       </c>
@@ -6887,7 +6907,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="67" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>91</v>
       </c>
@@ -6937,7 +6957,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="68" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>91</v>
       </c>
@@ -6987,7 +7007,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="69" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>91</v>
       </c>
@@ -7037,7 +7057,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>91</v>
       </c>
@@ -7087,7 +7107,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="71" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>91</v>
       </c>
@@ -7138,7 +7158,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="72" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>91</v>
       </c>
@@ -7189,7 +7209,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="73" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:16" x14ac:dyDescent="0.2">
       <c r="E73" t="s">
         <v>440</v>
       </c>
@@ -7200,7 +7220,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="74" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:16" x14ac:dyDescent="0.2">
       <c r="E74" t="s">
         <v>440</v>
       </c>
@@ -7211,7 +7231,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="75" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:16" x14ac:dyDescent="0.2">
       <c r="E75" t="s">
         <v>440</v>
       </c>
@@ -7222,7 +7242,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:16" x14ac:dyDescent="0.2">
       <c r="E76" t="s">
         <v>440</v>
       </c>
@@ -7233,7 +7253,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="77" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:16" x14ac:dyDescent="0.2">
       <c r="E77" t="s">
         <v>133</v>
       </c>
@@ -7244,7 +7264,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="78" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:16" x14ac:dyDescent="0.2">
       <c r="E78" t="s">
         <v>133</v>
       </c>
@@ -7255,7 +7275,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="79" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:16" x14ac:dyDescent="0.2">
       <c r="E79" t="s">
         <v>134</v>
       </c>
@@ -7266,7 +7286,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="80" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:16" x14ac:dyDescent="0.2">
       <c r="E80" t="s">
         <v>134</v>
       </c>
@@ -7277,7 +7297,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="81" spans="5:15" x14ac:dyDescent="0.35">
+    <row r="81" spans="5:15" x14ac:dyDescent="0.2">
       <c r="E81" t="s">
         <v>135</v>
       </c>
@@ -7288,7 +7308,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="82" spans="5:15" x14ac:dyDescent="0.35">
+    <row r="82" spans="5:15" x14ac:dyDescent="0.2">
       <c r="E82" t="s">
         <v>136</v>
       </c>
@@ -7299,7 +7319,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="83" spans="5:15" x14ac:dyDescent="0.35">
+    <row r="83" spans="5:15" x14ac:dyDescent="0.2">
       <c r="E83" t="s">
         <v>135</v>
       </c>
@@ -7310,7 +7330,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="84" spans="5:15" x14ac:dyDescent="0.35">
+    <row r="84" spans="5:15" x14ac:dyDescent="0.2">
       <c r="E84" t="s">
         <v>136</v>
       </c>
@@ -7321,7 +7341,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="85" spans="5:15" x14ac:dyDescent="0.35">
+    <row r="85" spans="5:15" x14ac:dyDescent="0.2">
       <c r="E85" t="s">
         <v>137</v>
       </c>
@@ -7332,7 +7352,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="86" spans="5:15" x14ac:dyDescent="0.35">
+    <row r="86" spans="5:15" x14ac:dyDescent="0.2">
       <c r="E86" t="s">
         <v>53</v>
       </c>
@@ -7343,7 +7363,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="87" spans="5:15" x14ac:dyDescent="0.35">
+    <row r="87" spans="5:15" x14ac:dyDescent="0.2">
       <c r="E87" t="s">
         <v>53</v>
       </c>
@@ -7354,7 +7374,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="88" spans="5:15" x14ac:dyDescent="0.35">
+    <row r="88" spans="5:15" x14ac:dyDescent="0.2">
       <c r="E88" t="s">
         <v>53</v>
       </c>
@@ -7369,7 +7389,7 @@
         <v/>
       </c>
     </row>
-    <row r="89" spans="5:15" x14ac:dyDescent="0.35">
+    <row r="89" spans="5:15" x14ac:dyDescent="0.2">
       <c r="E89" t="s">
         <v>53</v>
       </c>
@@ -7384,7 +7404,7 @@
         <v/>
       </c>
     </row>
-    <row r="90" spans="5:15" x14ac:dyDescent="0.35">
+    <row r="90" spans="5:15" x14ac:dyDescent="0.2">
       <c r="E90" t="s">
         <v>138</v>
       </c>
@@ -7399,7 +7419,7 @@
         <v/>
       </c>
     </row>
-    <row r="91" spans="5:15" x14ac:dyDescent="0.35">
+    <row r="91" spans="5:15" x14ac:dyDescent="0.2">
       <c r="E91" t="s">
         <v>138</v>
       </c>
@@ -7414,7 +7434,7 @@
         <v/>
       </c>
     </row>
-    <row r="92" spans="5:15" x14ac:dyDescent="0.35">
+    <row r="92" spans="5:15" x14ac:dyDescent="0.2">
       <c r="E92" t="s">
         <v>138</v>
       </c>
@@ -7429,7 +7449,7 @@
         <v/>
       </c>
     </row>
-    <row r="93" spans="5:15" x14ac:dyDescent="0.35">
+    <row r="93" spans="5:15" x14ac:dyDescent="0.2">
       <c r="E93" t="s">
         <v>139</v>
       </c>
@@ -7444,7 +7464,7 @@
         <v/>
       </c>
     </row>
-    <row r="94" spans="5:15" x14ac:dyDescent="0.35">
+    <row r="94" spans="5:15" x14ac:dyDescent="0.2">
       <c r="E94" t="s">
         <v>140</v>
       </c>
@@ -7459,7 +7479,7 @@
         <v/>
       </c>
     </row>
-    <row r="95" spans="5:15" x14ac:dyDescent="0.35">
+    <row r="95" spans="5:15" x14ac:dyDescent="0.2">
       <c r="E95" t="s">
         <v>139</v>
       </c>
@@ -7474,7 +7494,7 @@
         <v/>
       </c>
     </row>
-    <row r="96" spans="5:15" x14ac:dyDescent="0.35">
+    <row r="96" spans="5:15" x14ac:dyDescent="0.2">
       <c r="E96" t="s">
         <v>140</v>
       </c>
@@ -7489,7 +7509,7 @@
         <v/>
       </c>
     </row>
-    <row r="97" spans="5:15" x14ac:dyDescent="0.35">
+    <row r="97" spans="5:15" x14ac:dyDescent="0.2">
       <c r="E97" t="s">
         <v>139</v>
       </c>
@@ -7504,7 +7524,7 @@
         <v/>
       </c>
     </row>
-    <row r="98" spans="5:15" x14ac:dyDescent="0.35">
+    <row r="98" spans="5:15" x14ac:dyDescent="0.2">
       <c r="E98" t="s">
         <v>140</v>
       </c>
@@ -7519,7 +7539,7 @@
         <v/>
       </c>
     </row>
-    <row r="99" spans="5:15" x14ac:dyDescent="0.35">
+    <row r="99" spans="5:15" x14ac:dyDescent="0.2">
       <c r="E99" t="s">
         <v>139</v>
       </c>
@@ -7534,7 +7554,7 @@
         <v/>
       </c>
     </row>
-    <row r="100" spans="5:15" x14ac:dyDescent="0.35">
+    <row r="100" spans="5:15" x14ac:dyDescent="0.2">
       <c r="E100" t="s">
         <v>140</v>
       </c>
@@ -7549,7 +7569,7 @@
         <v/>
       </c>
     </row>
-    <row r="101" spans="5:15" x14ac:dyDescent="0.35">
+    <row r="101" spans="5:15" x14ac:dyDescent="0.2">
       <c r="E101" t="s">
         <v>139</v>
       </c>
@@ -7564,7 +7584,7 @@
         <v/>
       </c>
     </row>
-    <row r="102" spans="5:15" x14ac:dyDescent="0.35">
+    <row r="102" spans="5:15" x14ac:dyDescent="0.2">
       <c r="E102" t="s">
         <v>140</v>
       </c>
@@ -7579,7 +7599,7 @@
         <v/>
       </c>
     </row>
-    <row r="103" spans="5:15" x14ac:dyDescent="0.35">
+    <row r="103" spans="5:15" x14ac:dyDescent="0.2">
       <c r="E103" t="s">
         <v>61</v>
       </c>
@@ -7594,7 +7614,7 @@
         <v/>
       </c>
     </row>
-    <row r="104" spans="5:15" x14ac:dyDescent="0.35">
+    <row r="104" spans="5:15" x14ac:dyDescent="0.2">
       <c r="E104" t="s">
         <v>61</v>
       </c>
@@ -7609,7 +7629,7 @@
         <v/>
       </c>
     </row>
-    <row r="105" spans="5:15" x14ac:dyDescent="0.35">
+    <row r="105" spans="5:15" x14ac:dyDescent="0.2">
       <c r="E105" t="s">
         <v>56</v>
       </c>
@@ -7624,7 +7644,7 @@
         <v/>
       </c>
     </row>
-    <row r="106" spans="5:15" x14ac:dyDescent="0.35">
+    <row r="106" spans="5:15" x14ac:dyDescent="0.2">
       <c r="E106" t="s">
         <v>57</v>
       </c>
@@ -7639,7 +7659,7 @@
         <v/>
       </c>
     </row>
-    <row r="107" spans="5:15" x14ac:dyDescent="0.35">
+    <row r="107" spans="5:15" x14ac:dyDescent="0.2">
       <c r="E107" t="s">
         <v>58</v>
       </c>
@@ -7654,7 +7674,7 @@
         <v/>
       </c>
     </row>
-    <row r="108" spans="5:15" x14ac:dyDescent="0.35">
+    <row r="108" spans="5:15" x14ac:dyDescent="0.2">
       <c r="E108" t="s">
         <v>59</v>
       </c>
@@ -7669,7 +7689,7 @@
         <v/>
       </c>
     </row>
-    <row r="109" spans="5:15" x14ac:dyDescent="0.35">
+    <row r="109" spans="5:15" x14ac:dyDescent="0.2">
       <c r="E109" t="s">
         <v>441</v>
       </c>
@@ -7684,7 +7704,7 @@
         <v/>
       </c>
     </row>
-    <row r="110" spans="5:15" x14ac:dyDescent="0.35">
+    <row r="110" spans="5:15" x14ac:dyDescent="0.2">
       <c r="M110" t="s">
         <v>442</v>
       </c>
@@ -7693,7 +7713,7 @@
         <v/>
       </c>
     </row>
-    <row r="111" spans="5:15" x14ac:dyDescent="0.35">
+    <row r="111" spans="5:15" x14ac:dyDescent="0.2">
       <c r="M111" t="s">
         <v>442</v>
       </c>
@@ -7702,7 +7722,7 @@
         <v/>
       </c>
     </row>
-    <row r="112" spans="5:15" x14ac:dyDescent="0.35">
+    <row r="112" spans="5:15" x14ac:dyDescent="0.2">
       <c r="M112" t="s">
         <v>442</v>
       </c>
@@ -7711,7 +7731,7 @@
         <v/>
       </c>
     </row>
-    <row r="113" spans="13:15" x14ac:dyDescent="0.35">
+    <row r="113" spans="13:15" x14ac:dyDescent="0.2">
       <c r="M113" t="s">
         <v>442</v>
       </c>
@@ -7720,67 +7740,67 @@
         <v/>
       </c>
     </row>
-    <row r="114" spans="13:15" x14ac:dyDescent="0.35">
+    <row r="114" spans="13:15" x14ac:dyDescent="0.2">
       <c r="O114" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
-    <row r="115" spans="13:15" x14ac:dyDescent="0.35">
+    <row r="115" spans="13:15" x14ac:dyDescent="0.2">
       <c r="O115" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
-    <row r="116" spans="13:15" x14ac:dyDescent="0.35">
+    <row r="116" spans="13:15" x14ac:dyDescent="0.2">
       <c r="O116" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
-    <row r="117" spans="13:15" x14ac:dyDescent="0.35">
+    <row r="117" spans="13:15" x14ac:dyDescent="0.2">
       <c r="O117" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
-    <row r="118" spans="13:15" x14ac:dyDescent="0.35">
+    <row r="118" spans="13:15" x14ac:dyDescent="0.2">
       <c r="O118" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
-    <row r="119" spans="13:15" x14ac:dyDescent="0.35">
+    <row r="119" spans="13:15" x14ac:dyDescent="0.2">
       <c r="O119" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
-    <row r="120" spans="13:15" x14ac:dyDescent="0.35">
+    <row r="120" spans="13:15" x14ac:dyDescent="0.2">
       <c r="O120" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
-    <row r="121" spans="13:15" x14ac:dyDescent="0.35">
+    <row r="121" spans="13:15" x14ac:dyDescent="0.2">
       <c r="O121" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
-    <row r="122" spans="13:15" x14ac:dyDescent="0.35">
+    <row r="122" spans="13:15" x14ac:dyDescent="0.2">
       <c r="O122" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
-    <row r="123" spans="13:15" x14ac:dyDescent="0.35">
+    <row r="123" spans="13:15" x14ac:dyDescent="0.2">
       <c r="O123" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
-    <row r="124" spans="13:15" x14ac:dyDescent="0.35">
+    <row r="124" spans="13:15" x14ac:dyDescent="0.2">
       <c r="O124" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -7792,104 +7812,104 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:W39"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.453125" customWidth="1"/>
+    <col min="1" max="1" width="10.5" customWidth="1"/>
     <col min="2" max="2" width="8" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="14.26953125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.7265625" customWidth="1"/>
+    <col min="3" max="3" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.6640625" customWidth="1"/>
     <col min="7" max="7" width="18" customWidth="1"/>
-    <col min="8" max="8" width="18.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="26.6328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="53.26953125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="53.26953125" customWidth="1"/>
-    <col min="12" max="12" width="6.81640625" customWidth="1"/>
-    <col min="13" max="13" width="12.36328125" customWidth="1"/>
-    <col min="14" max="14" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="26.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="53.33203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="53.33203125" customWidth="1"/>
+    <col min="12" max="12" width="6.83203125" customWidth="1"/>
+    <col min="13" max="13" width="12.33203125" customWidth="1"/>
+    <col min="14" max="14" width="12.5" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="8" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="24.08984375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="11.6328125" customWidth="1"/>
-    <col min="18" max="20" width="12.36328125" customWidth="1"/>
-    <col min="21" max="21" width="15.6328125" customWidth="1"/>
-    <col min="22" max="22" width="14.90625" customWidth="1"/>
-    <col min="23" max="23" width="16.7265625" customWidth="1"/>
+    <col min="16" max="16" width="24.1640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.6640625" customWidth="1"/>
+    <col min="18" max="20" width="12.33203125" customWidth="1"/>
+    <col min="21" max="21" width="15.6640625" customWidth="1"/>
+    <col min="22" max="22" width="14.83203125" customWidth="1"/>
+    <col min="23" max="23" width="16.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" s="4" customFormat="1" ht="29" x14ac:dyDescent="0.35">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:23" s="3" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>251</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="L1" s="2" t="s">
         <v>296</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="M1" s="2" t="s">
         <v>297</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="N1" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="O1" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="P1" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="Q1" s="2" t="s">
         <v>298</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="R1" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="S1" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="T1" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="U1" s="3" t="s">
+      <c r="U1" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="V1" s="3" t="s">
+      <c r="V1" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="W1" s="3" t="s">
+      <c r="W1" s="2" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -7942,7 +7962,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -7995,7 +8015,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
@@ -8048,7 +8068,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
@@ -8101,7 +8121,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
@@ -8154,7 +8174,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>6</v>
       </c>
@@ -8207,7 +8227,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>7</v>
       </c>
@@ -8260,7 +8280,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>8</v>
       </c>
@@ -8313,7 +8333,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>9</v>
       </c>
@@ -8366,7 +8386,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>10</v>
       </c>
@@ -8419,7 +8439,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>11</v>
       </c>
@@ -8472,7 +8492,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>12</v>
       </c>
@@ -8525,7 +8545,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>13</v>
       </c>
@@ -8578,7 +8598,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>14</v>
       </c>
@@ -8631,7 +8651,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>15</v>
       </c>
@@ -8684,7 +8704,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>16</v>
       </c>
@@ -8737,7 +8757,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>17</v>
       </c>
@@ -8790,7 +8810,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>18</v>
       </c>
@@ -8843,7 +8863,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>19</v>
       </c>
@@ -8896,7 +8916,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>20</v>
       </c>
@@ -8949,7 +8969,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>21</v>
       </c>
@@ -9002,7 +9022,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>22</v>
       </c>
@@ -9055,7 +9075,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>23</v>
       </c>
@@ -9108,7 +9128,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>24</v>
       </c>
@@ -9161,7 +9181,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>25</v>
       </c>
@@ -9214,7 +9234,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>26</v>
       </c>
@@ -9267,7 +9287,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>27</v>
       </c>
@@ -9320,7 +9340,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>28</v>
       </c>
@@ -9373,7 +9393,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>29</v>
       </c>
@@ -9426,7 +9446,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>30</v>
       </c>
@@ -9479,7 +9499,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>31</v>
       </c>
@@ -9532,7 +9552,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>32</v>
       </c>
@@ -9585,7 +9605,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>33</v>
       </c>
@@ -9638,7 +9658,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>34</v>
       </c>
@@ -9691,7 +9711,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>35</v>
       </c>
@@ -9744,7 +9764,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>36</v>
       </c>
@@ -9797,7 +9817,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>37</v>
       </c>
@@ -9850,7 +9870,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>38</v>
       </c>
@@ -9909,84 +9929,84 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:W44"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.7265625" customWidth="1"/>
-    <col min="5" max="5" width="17.54296875" customWidth="1"/>
-    <col min="6" max="7" width="18.81640625" customWidth="1"/>
-    <col min="8" max="8" width="18.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="26.6328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="54.36328125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="54.36328125" customWidth="1"/>
-    <col min="12" max="12" width="6.90625" customWidth="1"/>
-    <col min="13" max="13" width="11.7265625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.6640625" customWidth="1"/>
+    <col min="5" max="5" width="17.5" customWidth="1"/>
+    <col min="6" max="7" width="18.83203125" customWidth="1"/>
+    <col min="8" max="8" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="26.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="54.33203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="54.33203125" customWidth="1"/>
+    <col min="12" max="12" width="6.83203125" customWidth="1"/>
+    <col min="13" max="13" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.5" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="8" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="25.90625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="5.7265625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="7.54296875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="25.83203125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.83203125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="7.5" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="12" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="15" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="15.1796875" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="17.08984375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="15.1640625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="17.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="29" x14ac:dyDescent="0.35">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:23" ht="48" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>251</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="L1" s="2" t="s">
         <v>296</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="M1" s="2" t="s">
         <v>297</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="N1" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="O1" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="P1" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="Q1" s="2" t="s">
         <v>298</v>
       </c>
       <c r="R1" s="1" t="s">
@@ -10008,7 +10028,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -10061,7 +10081,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -10114,7 +10134,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
@@ -10167,7 +10187,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
@@ -10220,7 +10240,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
@@ -10273,7 +10293,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>6</v>
       </c>
@@ -10326,484 +10346,484 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:23" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" t="s">
         <v>185</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" t="s">
         <v>5</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" t="s">
         <v>180</v>
       </c>
       <c r="E8" t="s">
         <v>250</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F8" t="s">
         <v>181</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="G8" t="s">
         <v>299</v>
       </c>
-      <c r="H8" s="2" t="s">
+      <c r="H8" t="s">
         <v>182</v>
       </c>
-      <c r="I8" s="2" t="s">
+      <c r="I8" t="s">
         <v>183</v>
       </c>
-      <c r="J8" s="2" t="s">
+      <c r="J8" t="s">
         <v>109</v>
       </c>
-      <c r="K8" s="2" t="s">
+      <c r="K8" t="s">
         <v>310</v>
       </c>
-      <c r="L8" s="2" t="s">
+      <c r="L8" t="s">
         <v>184</v>
       </c>
       <c r="M8" t="s">
         <v>347</v>
       </c>
-      <c r="N8" s="2">
+      <c r="N8">
         <v>300000</v>
       </c>
-      <c r="O8" s="2" t="s">
+      <c r="O8" t="s">
         <v>174</v>
       </c>
-      <c r="P8" s="2" t="s">
+      <c r="P8" t="s">
         <v>179</v>
       </c>
-      <c r="Q8" s="2" t="b">
+      <c r="Q8" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:23" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>8</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" t="s">
         <v>185</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" t="s">
         <v>5</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" t="s">
         <v>180</v>
       </c>
       <c r="E9" t="s">
         <v>250</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="F9" t="s">
         <v>181</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="G9" t="s">
         <v>299</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="H9" t="s">
         <v>182</v>
       </c>
-      <c r="I9" s="2" t="s">
+      <c r="I9" t="s">
         <v>183</v>
       </c>
-      <c r="J9" s="2" t="s">
+      <c r="J9" t="s">
         <v>110</v>
       </c>
-      <c r="K9" s="2" t="s">
+      <c r="K9" t="s">
         <v>311</v>
       </c>
-      <c r="L9" s="2" t="s">
+      <c r="L9" t="s">
         <v>184</v>
       </c>
       <c r="M9" t="s">
         <v>347</v>
       </c>
-      <c r="N9" s="2">
+      <c r="N9">
         <v>300000</v>
       </c>
-      <c r="O9" s="2" t="s">
+      <c r="O9" t="s">
         <v>174</v>
       </c>
-      <c r="P9" s="2" t="s">
+      <c r="P9" t="s">
         <v>179</v>
       </c>
-      <c r="Q9" s="2" t="b">
+      <c r="Q9" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:23" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>9</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" t="s">
         <v>185</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" t="s">
         <v>7</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" t="s">
         <v>180</v>
       </c>
       <c r="E10" t="s">
         <v>250</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="F10" t="s">
         <v>181</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="G10" t="s">
         <v>299</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="H10" t="s">
         <v>300</v>
       </c>
-      <c r="I10" s="2" t="s">
+      <c r="I10" t="s">
         <v>301</v>
       </c>
-      <c r="J10" s="2" t="s">
+      <c r="J10" t="s">
         <v>111</v>
       </c>
-      <c r="K10" s="2" t="s">
+      <c r="K10" t="s">
         <v>312</v>
       </c>
-      <c r="L10" s="2" t="s">
+      <c r="L10" t="s">
         <v>184</v>
       </c>
       <c r="M10" t="s">
         <v>347</v>
       </c>
-      <c r="N10" s="2">
+      <c r="N10">
         <v>150000</v>
       </c>
-      <c r="O10" s="2" t="s">
+      <c r="O10" t="s">
         <v>174</v>
       </c>
-      <c r="P10" s="2" t="s">
+      <c r="P10" t="s">
         <v>179</v>
       </c>
-      <c r="Q10" s="2" t="b">
+      <c r="Q10" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:23" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>10</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" t="s">
         <v>185</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" t="s">
         <v>7</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" t="s">
         <v>180</v>
       </c>
       <c r="E11" t="s">
         <v>250</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="F11" t="s">
         <v>181</v>
       </c>
-      <c r="G11" s="2" t="s">
+      <c r="G11" t="s">
         <v>299</v>
       </c>
-      <c r="H11" s="2" t="s">
+      <c r="H11" t="s">
         <v>300</v>
       </c>
-      <c r="I11" s="2" t="s">
+      <c r="I11" t="s">
         <v>301</v>
       </c>
-      <c r="J11" s="2" t="s">
+      <c r="J11" t="s">
         <v>33</v>
       </c>
-      <c r="K11" s="2" t="s">
+      <c r="K11" t="s">
         <v>267</v>
       </c>
-      <c r="L11" s="2" t="s">
+      <c r="L11" t="s">
         <v>184</v>
       </c>
       <c r="M11" t="s">
         <v>347</v>
       </c>
-      <c r="N11" s="2">
+      <c r="N11">
         <v>150000</v>
       </c>
-      <c r="O11" s="2" t="s">
+      <c r="O11" t="s">
         <v>174</v>
       </c>
-      <c r="P11" s="2" t="s">
+      <c r="P11" t="s">
         <v>179</v>
       </c>
-      <c r="Q11" s="2" t="b">
+      <c r="Q11" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:23" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>11</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" t="s">
         <v>185</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" t="s">
         <v>7</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D12" t="s">
         <v>180</v>
       </c>
       <c r="E12" t="s">
         <v>250</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="F12" t="s">
         <v>181</v>
       </c>
-      <c r="G12" s="2" t="s">
+      <c r="G12" t="s">
         <v>299</v>
       </c>
-      <c r="H12" s="2" t="s">
+      <c r="H12" t="s">
         <v>308</v>
       </c>
       <c r="I12" t="s">
         <v>304</v>
       </c>
-      <c r="J12" s="2" t="s">
+      <c r="J12" t="s">
         <v>112</v>
       </c>
-      <c r="K12" s="2" t="s">
+      <c r="K12" t="s">
         <v>313</v>
       </c>
-      <c r="L12" s="2" t="s">
+      <c r="L12" t="s">
         <v>184</v>
       </c>
       <c r="M12" t="s">
         <v>347</v>
       </c>
-      <c r="N12" s="2">
+      <c r="N12">
         <v>150000</v>
       </c>
-      <c r="O12" s="2" t="s">
+      <c r="O12" t="s">
         <v>174</v>
       </c>
-      <c r="P12" s="2" t="s">
+      <c r="P12" t="s">
         <v>179</v>
       </c>
-      <c r="Q12" s="2" t="b">
+      <c r="Q12" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:23" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>12</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" t="s">
         <v>185</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" t="s">
         <v>7</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="D13" t="s">
         <v>180</v>
       </c>
       <c r="E13" t="s">
         <v>250</v>
       </c>
-      <c r="F13" s="2" t="s">
+      <c r="F13" t="s">
         <v>181</v>
       </c>
-      <c r="G13" s="2" t="s">
+      <c r="G13" t="s">
         <v>299</v>
       </c>
-      <c r="H13" s="2" t="s">
+      <c r="H13" t="s">
         <v>308</v>
       </c>
       <c r="I13" t="s">
         <v>304</v>
       </c>
-      <c r="J13" s="2" t="s">
+      <c r="J13" t="s">
         <v>113</v>
       </c>
-      <c r="K13" s="2" t="s">
+      <c r="K13" t="s">
         <v>314</v>
       </c>
-      <c r="L13" s="2" t="s">
+      <c r="L13" t="s">
         <v>184</v>
       </c>
       <c r="M13" t="s">
         <v>347</v>
       </c>
-      <c r="N13" s="2">
+      <c r="N13">
         <v>150000</v>
       </c>
-      <c r="O13" s="2" t="s">
+      <c r="O13" t="s">
         <v>174</v>
       </c>
-      <c r="P13" s="2" t="s">
+      <c r="P13" t="s">
         <v>179</v>
       </c>
-      <c r="Q13" s="2" t="b">
+      <c r="Q13" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:23" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>13</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" t="s">
         <v>185</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" t="s">
         <v>13</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="D14" t="s">
         <v>180</v>
       </c>
       <c r="E14" t="s">
         <v>250</v>
       </c>
-      <c r="F14" s="2" t="s">
+      <c r="F14" t="s">
         <v>181</v>
       </c>
-      <c r="G14" s="2" t="s">
+      <c r="G14" t="s">
         <v>299</v>
       </c>
-      <c r="H14" s="2" t="s">
+      <c r="H14" t="s">
         <v>308</v>
       </c>
       <c r="I14" t="s">
         <v>304</v>
       </c>
-      <c r="J14" s="2" t="s">
+      <c r="J14" t="s">
         <v>114</v>
       </c>
-      <c r="K14" s="2" t="s">
+      <c r="K14" t="s">
         <v>315</v>
       </c>
-      <c r="L14" s="2" t="s">
+      <c r="L14" t="s">
         <v>184</v>
       </c>
       <c r="M14" t="s">
         <v>347</v>
       </c>
-      <c r="N14" s="2">
+      <c r="N14">
         <v>250000</v>
       </c>
-      <c r="O14" s="2" t="s">
+      <c r="O14" t="s">
         <v>174</v>
       </c>
-      <c r="P14" s="2" t="s">
+      <c r="P14" t="s">
         <v>179</v>
       </c>
-      <c r="Q14" s="2" t="b">
+      <c r="Q14" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:23" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>14</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" t="s">
         <v>185</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C15" t="s">
         <v>94</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="D15" t="s">
         <v>180</v>
       </c>
       <c r="E15" t="s">
         <v>250</v>
       </c>
-      <c r="F15" s="2" t="s">
+      <c r="F15" t="s">
         <v>181</v>
       </c>
-      <c r="G15" s="2" t="s">
+      <c r="G15" t="s">
         <v>299</v>
       </c>
-      <c r="H15" s="2" t="s">
+      <c r="H15" t="s">
         <v>303</v>
       </c>
       <c r="I15" t="s">
         <v>305</v>
       </c>
-      <c r="J15" s="2" t="s">
+      <c r="J15" t="s">
         <v>37</v>
       </c>
-      <c r="K15" s="2" t="s">
+      <c r="K15" t="s">
         <v>316</v>
       </c>
-      <c r="L15" s="2" t="s">
+      <c r="L15" t="s">
         <v>184</v>
       </c>
       <c r="M15" t="s">
         <v>347</v>
       </c>
-      <c r="N15" s="2">
+      <c r="N15">
         <v>200000</v>
       </c>
-      <c r="O15" s="2" t="s">
+      <c r="O15" t="s">
         <v>174</v>
       </c>
-      <c r="P15" s="2" t="s">
+      <c r="P15" t="s">
         <v>179</v>
       </c>
-      <c r="Q15" s="2" t="b">
+      <c r="Q15" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:23" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>15</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" t="s">
         <v>185</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" t="s">
         <v>94</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="D16" t="s">
         <v>180</v>
       </c>
       <c r="E16" t="s">
         <v>250</v>
       </c>
-      <c r="F16" s="2" t="s">
+      <c r="F16" t="s">
         <v>181</v>
       </c>
-      <c r="G16" s="2" t="s">
+      <c r="G16" t="s">
         <v>299</v>
       </c>
-      <c r="H16" s="2" t="s">
+      <c r="H16" t="s">
         <v>303</v>
       </c>
       <c r="I16" t="s">
         <v>305</v>
       </c>
-      <c r="J16" s="2" t="s">
+      <c r="J16" t="s">
         <v>229</v>
       </c>
-      <c r="K16" s="2" t="s">
+      <c r="K16" t="s">
         <v>317</v>
       </c>
-      <c r="L16" s="2" t="s">
+      <c r="L16" t="s">
         <v>184</v>
       </c>
       <c r="M16" t="s">
         <v>347</v>
       </c>
-      <c r="N16" s="2">
+      <c r="N16">
         <v>200000</v>
       </c>
-      <c r="O16" s="2" t="s">
+      <c r="O16" t="s">
         <v>174</v>
       </c>
-      <c r="P16" s="2" t="s">
+      <c r="P16" t="s">
         <v>179</v>
       </c>
-      <c r="Q16" s="2" t="b">
+      <c r="Q16" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>16</v>
       </c>
@@ -10822,6 +10842,9 @@
       <c r="F17" t="s">
         <v>186</v>
       </c>
+      <c r="G17" t="s">
+        <v>247</v>
+      </c>
       <c r="H17" t="s">
         <v>187</v>
       </c>
@@ -10853,7 +10876,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>17</v>
       </c>
@@ -10872,6 +10895,9 @@
       <c r="F18" t="s">
         <v>186</v>
       </c>
+      <c r="G18" t="s">
+        <v>247</v>
+      </c>
       <c r="H18" t="s">
         <v>187</v>
       </c>
@@ -10903,7 +10929,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>18</v>
       </c>
@@ -10922,6 +10948,9 @@
       <c r="F19" t="s">
         <v>186</v>
       </c>
+      <c r="G19" t="s">
+        <v>247</v>
+      </c>
       <c r="H19" t="s">
         <v>187</v>
       </c>
@@ -10953,7 +10982,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>19</v>
       </c>
@@ -10972,6 +11001,9 @@
       <c r="F20" t="s">
         <v>186</v>
       </c>
+      <c r="G20" t="s">
+        <v>247</v>
+      </c>
       <c r="H20" t="s">
         <v>187</v>
       </c>
@@ -11003,7 +11035,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>20</v>
       </c>
@@ -11022,6 +11054,9 @@
       <c r="F21" t="s">
         <v>186</v>
       </c>
+      <c r="G21" t="s">
+        <v>247</v>
+      </c>
       <c r="H21" t="s">
         <v>195</v>
       </c>
@@ -11053,7 +11088,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>21</v>
       </c>
@@ -11072,6 +11107,9 @@
       <c r="F22" t="s">
         <v>186</v>
       </c>
+      <c r="G22" t="s">
+        <v>247</v>
+      </c>
       <c r="H22" t="s">
         <v>195</v>
       </c>
@@ -11103,7 +11141,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>22</v>
       </c>
@@ -11122,6 +11160,9 @@
       <c r="F23" t="s">
         <v>186</v>
       </c>
+      <c r="G23" t="s">
+        <v>247</v>
+      </c>
       <c r="H23" t="s">
         <v>195</v>
       </c>
@@ -11153,7 +11194,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>23</v>
       </c>
@@ -11172,6 +11213,9 @@
       <c r="F24" t="s">
         <v>186</v>
       </c>
+      <c r="G24" t="s">
+        <v>247</v>
+      </c>
       <c r="H24" t="s">
         <v>195</v>
       </c>
@@ -11203,7 +11247,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>24</v>
       </c>
@@ -11222,6 +11266,9 @@
       <c r="F25" t="s">
         <v>186</v>
       </c>
+      <c r="G25" t="s">
+        <v>247</v>
+      </c>
       <c r="H25" t="s">
         <v>199</v>
       </c>
@@ -11253,7 +11300,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>25</v>
       </c>
@@ -11272,6 +11319,9 @@
       <c r="F26" t="s">
         <v>186</v>
       </c>
+      <c r="G26" t="s">
+        <v>247</v>
+      </c>
       <c r="H26" t="s">
         <v>199</v>
       </c>
@@ -11303,7 +11353,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>26</v>
       </c>
@@ -11322,6 +11372,9 @@
       <c r="F27" t="s">
         <v>186</v>
       </c>
+      <c r="G27" t="s">
+        <v>247</v>
+      </c>
       <c r="H27" t="s">
         <v>202</v>
       </c>
@@ -11353,7 +11406,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>27</v>
       </c>
@@ -11372,6 +11425,9 @@
       <c r="F28" t="s">
         <v>186</v>
       </c>
+      <c r="G28" t="s">
+        <v>247</v>
+      </c>
       <c r="H28" t="s">
         <v>202</v>
       </c>
@@ -11403,7 +11459,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>28</v>
       </c>
@@ -11422,6 +11478,9 @@
       <c r="F29" t="s">
         <v>208</v>
       </c>
+      <c r="G29" t="s">
+        <v>248</v>
+      </c>
       <c r="H29" t="s">
         <v>209</v>
       </c>
@@ -11453,7 +11512,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>29</v>
       </c>
@@ -11472,6 +11531,9 @@
       <c r="F30" t="s">
         <v>208</v>
       </c>
+      <c r="G30" t="s">
+        <v>248</v>
+      </c>
       <c r="H30" t="s">
         <v>209</v>
       </c>
@@ -11503,7 +11565,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>30</v>
       </c>
@@ -11522,6 +11584,9 @@
       <c r="F31" t="s">
         <v>208</v>
       </c>
+      <c r="G31" t="s">
+        <v>248</v>
+      </c>
       <c r="H31" t="s">
         <v>209</v>
       </c>
@@ -11553,7 +11618,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>31</v>
       </c>
@@ -11572,6 +11637,9 @@
       <c r="F32" t="s">
         <v>208</v>
       </c>
+      <c r="G32" t="s">
+        <v>248</v>
+      </c>
       <c r="H32" t="s">
         <v>209</v>
       </c>
@@ -11603,7 +11671,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>32</v>
       </c>
@@ -11622,6 +11690,9 @@
       <c r="F33" t="s">
         <v>208</v>
       </c>
+      <c r="G33" t="s">
+        <v>248</v>
+      </c>
       <c r="H33" t="s">
         <v>209</v>
       </c>
@@ -11653,7 +11724,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>33</v>
       </c>
@@ -11672,6 +11743,9 @@
       <c r="F34" t="s">
         <v>208</v>
       </c>
+      <c r="G34" t="s">
+        <v>248</v>
+      </c>
       <c r="H34" t="s">
         <v>216</v>
       </c>
@@ -11684,10 +11758,10 @@
       <c r="K34" t="s">
         <v>334</v>
       </c>
-      <c r="L34" s="2" t="s">
+      <c r="L34" t="s">
         <v>190</v>
       </c>
-      <c r="M34" s="2" t="s">
+      <c r="M34" t="s">
         <v>191</v>
       </c>
       <c r="N34">
@@ -11703,7 +11777,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>34</v>
       </c>
@@ -11722,6 +11796,9 @@
       <c r="F35" t="s">
         <v>208</v>
       </c>
+      <c r="G35" t="s">
+        <v>248</v>
+      </c>
       <c r="H35" t="s">
         <v>216</v>
       </c>
@@ -11753,7 +11830,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>35</v>
       </c>
@@ -11772,6 +11849,9 @@
       <c r="F36" t="s">
         <v>208</v>
       </c>
+      <c r="G36" t="s">
+        <v>248</v>
+      </c>
       <c r="H36" t="s">
         <v>216</v>
       </c>
@@ -11803,7 +11883,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>36</v>
       </c>
@@ -11822,6 +11902,9 @@
       <c r="F37" t="s">
         <v>208</v>
       </c>
+      <c r="G37" t="s">
+        <v>248</v>
+      </c>
       <c r="H37" t="s">
         <v>216</v>
       </c>
@@ -11853,7 +11936,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>37</v>
       </c>
@@ -11872,6 +11955,9 @@
       <c r="F38" t="s">
         <v>208</v>
       </c>
+      <c r="G38" t="s">
+        <v>248</v>
+      </c>
       <c r="H38" t="s">
         <v>216</v>
       </c>
@@ -11903,7 +11989,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>38</v>
       </c>
@@ -11922,6 +12008,9 @@
       <c r="F39" t="s">
         <v>208</v>
       </c>
+      <c r="G39" t="s">
+        <v>248</v>
+      </c>
       <c r="H39" t="s">
         <v>216</v>
       </c>
@@ -11953,7 +12042,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>39</v>
       </c>
@@ -11972,6 +12061,9 @@
       <c r="F40" t="s">
         <v>221</v>
       </c>
+      <c r="G40" t="s">
+        <v>295</v>
+      </c>
       <c r="H40" t="s">
         <v>222</v>
       </c>
@@ -12003,7 +12095,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>40</v>
       </c>
@@ -12022,6 +12114,9 @@
       <c r="F41" t="s">
         <v>221</v>
       </c>
+      <c r="G41" t="s">
+        <v>295</v>
+      </c>
       <c r="H41" t="s">
         <v>222</v>
       </c>
@@ -12053,7 +12148,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>41</v>
       </c>
@@ -12072,6 +12167,9 @@
       <c r="F42" t="s">
         <v>221</v>
       </c>
+      <c r="G42" t="s">
+        <v>295</v>
+      </c>
       <c r="H42" t="s">
         <v>177</v>
       </c>
@@ -12103,7 +12201,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>42</v>
       </c>
@@ -12122,6 +12220,9 @@
       <c r="F43" t="s">
         <v>221</v>
       </c>
+      <c r="G43" t="s">
+        <v>295</v>
+      </c>
       <c r="H43" t="s">
         <v>226</v>
       </c>
@@ -12153,7 +12254,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>43</v>
       </c>
@@ -12171,6 +12272,9 @@
       </c>
       <c r="F44" t="s">
         <v>221</v>
+      </c>
+      <c r="G44" t="s">
+        <v>295</v>
       </c>
       <c r="H44" t="s">
         <v>227</v>

</xml_diff>